<commit_message>
test: perbarui rekap hasil pengujian wajib
Sederhanakan benchmark ke kategori wajib dan perbarui artefak hasil JSON serta XLSX.
</commit_message>
<xml_diff>
--- a/data-uji/hasil/hasil-pengujian.xlsx
+++ b/data-uji/hasil/hasil-pengujian.xlsx
@@ -12,14 +12,13 @@
     <sheet sheetId="6" name="4 Uji tamper" state="visible" r:id="rId9"/>
     <sheet sheetId="7" name="5 Uji kunci salah" state="visible" r:id="rId10"/>
     <sheet sheetId="8" name="6 Uji QR-Code palsu" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="7 Beberapa penandatangan" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="73">
   <si>
     <t>Kunci privat tidak pernah ditulis polos: hanya bentuk terenkripsi (PKCS#8 dalam AES-256-GCM, kunci dari kata sandi dengan scrypt) yang disimpan.</t>
   </si>
@@ -96,7 +95,7 @@
     <t>Payload QR-Code (B)</t>
   </si>
   <si>
-    <t>versi 13, 69x69 modul, koreksi kesalahan M</t>
+    <t>versi 14, 73x73 modul, koreksi kesalahan M</t>
   </si>
   <si>
     <t>PDF asli (3 halaman)</t>
@@ -105,10 +104,10 @@
     <t>PDF setelah halaman QR dan 1 blok</t>
   </si>
   <si>
-    <t>tambahan 15076 B</t>
-  </si>
-  <si>
-    <t>Setiap baris memakai lebih dari 30 ulangan (200). Node v24.17.0.</t>
+    <t>tambahan 16520 B</t>
+  </si>
+  <si>
+    <t>Setiap baris memakai lebih dari 30 ulangan (200). Node v24.13.0.</t>
   </si>
   <si>
     <t>ECDSA sign (pesan pendek)</t>
@@ -174,52 +173,25 @@
     <t>PDF 20 halaman (43181 B)</t>
   </si>
   <si>
-    <t>Isi dokumen: 1 bit dibalik pada hingga 400 posisi tersebar (semua posisi untuk berkas kecil). Blok tanda tangan: 1 bit dibalik pada setiap byte blok. Target: 100% terdeteksi.</t>
+    <t>Satu byte pada isi dokumen bertanda tangan diubah. Verifikasi wajib menolak hasil perubahan.</t>
   </si>
   <si>
     <t>Ukuran bertanda tangan (B)</t>
   </si>
   <si>
-    <t>Ubah 1 bit isi dokumen: terdeteksi</t>
-  </si>
-  <si>
-    <t>Ubah 1 bit di blok tanda tangan: terdeteksi</t>
-  </si>
-  <si>
-    <t>Tambah, potong, awalan: terdeteksi</t>
-  </si>
-  <si>
-    <t>Berkas asli</t>
-  </si>
-  <si>
-    <t>PDF 1 halaman</t>
-  </si>
-  <si>
-    <t>400 dari 400</t>
-  </si>
-  <si>
-    <t>693 dari 693</t>
-  </si>
-  <si>
-    <t>3 dari 3</t>
-  </si>
-  <si>
-    <t>sah</t>
-  </si>
-  <si>
-    <t>PDF 5 halaman</t>
-  </si>
-  <si>
-    <t>PDF 20 halaman</t>
-  </si>
-  <si>
-    <t>teks 2 KB</t>
-  </si>
-  <si>
-    <t>teks pendek</t>
-  </si>
-  <si>
-    <t>18 dari 18</t>
+    <t>Perubahan</t>
+  </si>
+  <si>
+    <t>Hasil verifikasi</t>
+  </si>
+  <si>
+    <t>PDF 3 halaman</t>
+  </si>
+  <si>
+    <t>1 byte isi dokumen diubah</t>
+  </si>
+  <si>
+    <t>ditolak</t>
   </si>
   <si>
     <t>Kunci publik yang tidak cocok menghasilkan kegagalan. Nama yang sama tidak berarti kunci yang sama: identitas dinilai dari sidik jari kunci terdaftar.</t>
@@ -231,39 +203,21 @@
     <t>Hasil</t>
   </si>
   <si>
-    <t>Kunci publik acak lain (50 kunci)</t>
-  </si>
-  <si>
-    <t>50 dari 50 ditolak</t>
-  </si>
-  <si>
-    <t>Kunci publik penandatangan</t>
+    <t>Kunci publik yang salah</t>
+  </si>
+  <si>
+    <t>Kunci publik yang benar</t>
   </si>
   <si>
     <t>diterima</t>
   </si>
   <si>
-    <t>Penipu memakai nama yang sama dengan kunci sendiri: tanda tangan sah secara matematis</t>
-  </si>
-  <si>
-    <t>ya</t>
-  </si>
-  <si>
-    <t>... tetapi kunci terdaftar</t>
-  </si>
-  <si>
-    <t>TIDAK TERDAFTAR</t>
-  </si>
-  <si>
-    <t>Payload QR 320 B (versi 13, 69x69 modul). QR memuat metadata dan tanda tangan atas metadata + ID dokumen; QR sah saja tidak membuktikan isi dokumen, itu tugas tanda tangan dokumen.</t>
+    <t>Payload QR 348 B (versi 14, 73x73 modul). QR memuat metadata dan tanda tangan atas metadata + ID dokumen; QR sah saja tidak membuktikan isi dokumen, itu tugas tanda tangan dokumen.</t>
   </si>
   <si>
     <t>nama diubah</t>
   </si>
   <si>
-    <t>ditolak</t>
-  </si>
-  <si>
     <t>jabatan diubah</t>
   </si>
   <si>
@@ -279,76 +233,10 @@
     <t>sidik jari diubah</t>
   </si>
   <si>
-    <t>tanda tangan di QR: 1 bit dibalik pada tiap byte (64 uji)</t>
-  </si>
-  <si>
-    <t>64 dari 64 ditolak</t>
-  </si>
-  <si>
-    <t>QR penandatangan lain ditempel</t>
-  </si>
-  <si>
-    <t>QR sah milik dokumen lain (penandatangan sama)</t>
-  </si>
-  <si>
-    <t>ditolak (ID dokumen tidak cocok)</t>
-  </si>
-  <si>
-    <t>teks QR bukan payload</t>
+    <t>Signature pada QR diubah</t>
   </si>
   <si>
     <t>QR asli</t>
-  </si>
-  <si>
-    <t>Setiap penandatangan menambah satu blok yang menandatangani semua yang ada sebelumnya. Mengubah dokumen membatalkan semua tanda tangan; menghapus penandatangan terakhir meninggalkan yang sebelumnya tetap sah.</t>
-  </si>
-  <si>
-    <t>Jumlah penandatangan</t>
-  </si>
-  <si>
-    <t>Ukuran berkas (B)</t>
-  </si>
-  <si>
-    <t>Tambahan dari 1 penandatangan (B)</t>
-  </si>
-  <si>
-    <t>Waktu verifikasi (ms)</t>
-  </si>
-  <si>
-    <t>Berkas utuh</t>
-  </si>
-  <si>
-    <t>Satu bit isi diubah</t>
-  </si>
-  <si>
-    <t>1 dari 1 sah</t>
-  </si>
-  <si>
-    <t>1 dari 1 ditolak</t>
-  </si>
-  <si>
-    <t>2 dari 2 sah</t>
-  </si>
-  <si>
-    <t>2 dari 2 ditolak</t>
-  </si>
-  <si>
-    <t>3 dari 3 sah</t>
-  </si>
-  <si>
-    <t>3 dari 3 ditolak</t>
-  </si>
-  <si>
-    <t>4 dari 4 sah</t>
-  </si>
-  <si>
-    <t>4 dari 4 ditolak</t>
-  </si>
-  <si>
-    <t>5 dari 5 sah</t>
-  </si>
-  <si>
-    <t>5 dari 5 ditolak</t>
   </si>
 </sst>
 </file>
@@ -768,16 +656,16 @@
         <v>100</v>
       </c>
       <c r="C4">
-        <v>0.0289</v>
+        <v>0.0661</v>
       </c>
       <c r="D4">
-        <v>0.053</v>
+        <v>0.1053</v>
       </c>
       <c r="E4">
-        <v>0.02</v>
+        <v>0.0452</v>
       </c>
       <c r="F4">
-        <v>0.5532</v>
+        <v>1.1072</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -788,16 +676,16 @@
         <v>30</v>
       </c>
       <c r="C5">
-        <v>49.8281</v>
+        <v>93.4608</v>
       </c>
       <c r="D5">
-        <v>0.8324</v>
+        <v>8.2538</v>
       </c>
       <c r="E5">
-        <v>48.6564</v>
+        <v>83.5164</v>
       </c>
       <c r="F5">
-        <v>52.0859</v>
+        <v>110.6431</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -808,16 +696,16 @@
         <v>30</v>
       </c>
       <c r="C6">
-        <v>50.0142</v>
+        <v>86.2643</v>
       </c>
       <c r="D6">
-        <v>0.9217</v>
+        <v>1.4538</v>
       </c>
       <c r="E6">
-        <v>48.531</v>
+        <v>83.9627</v>
       </c>
       <c r="F6">
-        <v>51.9582</v>
+        <v>90.7084</v>
       </c>
     </row>
   </sheetData>
@@ -916,7 +804,7 @@
         <v>24</v>
       </c>
       <c r="B8">
-        <v>320</v>
+        <v>348</v>
       </c>
       <c r="C8" t="s">
         <v>25</v>
@@ -938,7 +826,7 @@
         <v>27</v>
       </c>
       <c r="B10">
-        <v>22281</v>
+        <v>23725</v>
       </c>
       <c r="C10" t="s">
         <v>28</v>
@@ -991,16 +879,16 @@
         <v>200</v>
       </c>
       <c r="C4">
-        <v>0.0224</v>
+        <v>0.0575</v>
       </c>
       <c r="D4">
-        <v>0.0022</v>
+        <v>0.0342</v>
       </c>
       <c r="E4">
-        <v>0.0209</v>
+        <v>0.0409</v>
       </c>
       <c r="F4">
-        <v>0.036</v>
+        <v>0.3738</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1011,16 +899,16 @@
         <v>200</v>
       </c>
       <c r="C5">
-        <v>0.0544</v>
+        <v>0.1139</v>
       </c>
       <c r="D5">
-        <v>0.0027</v>
+        <v>0.0339</v>
       </c>
       <c r="E5">
-        <v>0.052</v>
+        <v>0.0821</v>
       </c>
       <c r="F5">
-        <v>0.0741</v>
+        <v>0.233</v>
       </c>
     </row>
   </sheetData>
@@ -1070,19 +958,19 @@
         <v>40</v>
       </c>
       <c r="B4">
-        <v>0.0021</v>
+        <v>0.0067</v>
       </c>
       <c r="C4">
-        <v>14.9255</v>
+        <v>31.1409</v>
       </c>
       <c r="D4">
-        <v>0.7935</v>
+        <v>1.4662</v>
       </c>
       <c r="E4">
-        <v>0.1796</v>
+        <v>0.4117</v>
       </c>
       <c r="F4">
-        <v>0.0358</v>
+        <v>0.1344</v>
       </c>
       <c r="G4">
         <v>40</v>
@@ -1093,19 +981,19 @@
         <v>41</v>
       </c>
       <c r="B5">
-        <v>0.0489</v>
+        <v>0.2322</v>
       </c>
       <c r="C5">
-        <v>15.1379</v>
+        <v>34.4761</v>
       </c>
       <c r="D5">
-        <v>1.0969</v>
+        <v>8.4333</v>
       </c>
       <c r="E5">
-        <v>0.2076</v>
+        <v>0.5882</v>
       </c>
       <c r="F5">
-        <v>0.0143</v>
+        <v>0.1627</v>
       </c>
       <c r="G5">
         <v>40</v>
@@ -1116,19 +1004,19 @@
         <v>42</v>
       </c>
       <c r="B6">
-        <v>0.5034</v>
+        <v>2.4234</v>
       </c>
       <c r="C6">
-        <v>15.8538</v>
+        <v>36.0842</v>
       </c>
       <c r="D6">
-        <v>1.1053</v>
+        <v>2.6726</v>
       </c>
       <c r="E6">
-        <v>0.6644</v>
+        <v>2.8186</v>
       </c>
       <c r="F6">
-        <v>0.0397</v>
+        <v>0.3276</v>
       </c>
       <c r="G6">
         <v>40</v>
@@ -1139,19 +1027,19 @@
         <v>43</v>
       </c>
       <c r="B7">
-        <v>4.882</v>
+        <v>23.9594</v>
       </c>
       <c r="C7">
-        <v>22.4869</v>
+        <v>62.6141</v>
       </c>
       <c r="D7">
-        <v>1.5546</v>
+        <v>4.8206</v>
       </c>
       <c r="E7">
-        <v>5.2908</v>
+        <v>25.2033</v>
       </c>
       <c r="F7">
-        <v>0.2549</v>
+        <v>0.9118</v>
       </c>
       <c r="G7">
         <v>30</v>
@@ -1198,16 +1086,16 @@
         <v>48</v>
       </c>
       <c r="B4">
-        <v>35.359</v>
+        <v>90.109</v>
       </c>
       <c r="C4">
-        <v>9.3171</v>
+        <v>21.2104</v>
       </c>
       <c r="D4">
-        <v>0.1804</v>
+        <v>0.7563</v>
       </c>
       <c r="E4">
-        <v>0.0182</v>
+        <v>0.3835</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -1215,16 +1103,16 @@
         <v>49</v>
       </c>
       <c r="B5">
-        <v>31.7578</v>
+        <v>125.9966</v>
       </c>
       <c r="C5">
-        <v>2.1623</v>
+        <v>46.4953</v>
       </c>
       <c r="D5">
-        <v>0.172</v>
+        <v>0.7401</v>
       </c>
       <c r="E5">
-        <v>0.0201</v>
+        <v>0.1208</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -1232,16 +1120,16 @@
         <v>50</v>
       </c>
       <c r="B6">
-        <v>42.189</v>
+        <v>95.2596</v>
       </c>
       <c r="C6">
-        <v>6.5488</v>
+        <v>12.1037</v>
       </c>
       <c r="D6">
-        <v>0.1948</v>
+        <v>0.6124</v>
       </c>
       <c r="E6">
-        <v>0.0381</v>
+        <v>0.2263</v>
       </c>
     </row>
   </sheetData>
@@ -1252,10 +1140,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="6" width="26" customWidth="1"/>
+    <col min="1" max="4" width="26" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
@@ -1263,7 +1151,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>45</v>
       </c>
@@ -1276,111 +1164,19 @@
       <c r="D3" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="1" t="s">
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>55</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="B4">
+        <v>23889</v>
+      </c>
+      <c r="C4" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="D4" t="s">
         <v>57</v>
-      </c>
-      <c r="B4">
-        <v>17991</v>
-      </c>
-      <c r="C4" t="s">
-        <v>58</v>
-      </c>
-      <c r="D4" t="s">
-        <v>59</v>
-      </c>
-      <c r="E4" t="s">
-        <v>60</v>
-      </c>
-      <c r="F4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>62</v>
-      </c>
-      <c r="B5">
-        <v>26349</v>
-      </c>
-      <c r="C5" t="s">
-        <v>58</v>
-      </c>
-      <c r="D5" t="s">
-        <v>59</v>
-      </c>
-      <c r="E5" t="s">
-        <v>60</v>
-      </c>
-      <c r="F5" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B6">
-        <v>58163</v>
-      </c>
-      <c r="C6" t="s">
-        <v>58</v>
-      </c>
-      <c r="D6" t="s">
-        <v>59</v>
-      </c>
-      <c r="E6" t="s">
-        <v>60</v>
-      </c>
-      <c r="F6" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7">
-        <v>2741</v>
-      </c>
-      <c r="C7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D7" t="s">
-        <v>59</v>
-      </c>
-      <c r="E7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F7" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>65</v>
-      </c>
-      <c r="B8">
-        <v>711</v>
-      </c>
-      <c r="C8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D8" t="s">
-        <v>59</v>
-      </c>
-      <c r="E8" t="s">
-        <v>60</v>
-      </c>
-      <c r="F8" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1391,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="26" customWidth="1"/>
@@ -1399,47 +1195,31 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>74</v>
-      </c>
-      <c r="B6" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>76</v>
-      </c>
-      <c r="B7" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -1450,7 +1230,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="26" customWidth="1"/>
@@ -1458,242 +1238,79 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>66</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>71</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>57</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B11" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B12" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>91</v>
-      </c>
-      <c r="B13" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B14" t="s">
-        <v>73</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F8"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="6" width="26" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4">
-        <v>1</v>
-      </c>
-      <c r="B4">
-        <v>20151</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0.1834</v>
-      </c>
-      <c r="E4" t="s">
-        <v>100</v>
-      </c>
-      <c r="F4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5">
-        <v>2</v>
-      </c>
-      <c r="B5">
-        <v>20831</v>
-      </c>
-      <c r="C5">
-        <v>680</v>
-      </c>
-      <c r="D5">
-        <v>0.3123</v>
-      </c>
-      <c r="E5" t="s">
-        <v>102</v>
-      </c>
-      <c r="F5" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>21511</v>
-      </c>
-      <c r="C6">
-        <v>1360</v>
-      </c>
-      <c r="D6">
-        <v>0.496</v>
-      </c>
-      <c r="E6" t="s">
-        <v>104</v>
-      </c>
-      <c r="F6" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7">
-        <v>4</v>
-      </c>
-      <c r="B7">
-        <v>22191</v>
-      </c>
-      <c r="C7">
-        <v>2040</v>
-      </c>
-      <c r="D7">
-        <v>0.6245</v>
-      </c>
-      <c r="E7" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <v>5</v>
-      </c>
-      <c r="B8">
-        <v>22871</v>
-      </c>
-      <c r="C8">
-        <v>2720</v>
-      </c>
-      <c r="D8">
-        <v>0.8771</v>
-      </c>
-      <c r="E8" t="s">
-        <v>108</v>
-      </c>
-      <c r="F8" t="s">
-        <v>109</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>